<commit_message>
Complete Task 26: validate cafe scene background convention
- Route 48 ordinary cafe conversation pages through scene.cafe\n- Preserve special cafe artwork aliases and verify explicit restoration\n- Record generation, Unity, and direct contract evidence\n\nProgress: 26/95 tasks (27%)\nTask Directory: .autonomous/ncs-formal-integration-overnight/
</commit_message>
<xml_diff>
--- a/Assets/ConfigTables/Data/Narrative/Narrative.xlsx
+++ b/Assets/ConfigTables/Data/Narrative/Narrative.xlsx
@@ -1,40 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Object" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Trigger" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Event" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="EventDate" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Result" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Condition" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Template" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="SetupParams" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Choice" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="OpeningPresentation" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="OpeningLine" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Action" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="MapPosition" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="PresentationIndex" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="ConversationPage" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ConversationLine" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Notice" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="ReadingPage" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="ReadingLine" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="ConditionKey" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="ActionMilestone" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Ending" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="CafeVisit" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="CafeVisitHook" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="AbilityCheck" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="AbilityCheckCondition" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="CafeTutorialStep" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trigger" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EventDate" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Result" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Condition" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SetupParams" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choice" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OpeningPresentation" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OpeningLine" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapPosition" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PresentationIndex" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ConversationPage" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ConversationLine" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notice" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadingPage" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadingLine" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ConditionKey" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActionMilestone" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ending" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CafeVisit" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CafeVisitHook" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AbilityCheck" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AbilityCheckCondition" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CafeTutorialStep" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4698,7 +4698,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4762,7 +4762,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4794,7 +4794,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4858,7 +4858,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -4890,7 +4890,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -5146,7 +5146,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -5178,7 +5178,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -5210,7 +5210,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -5242,7 +5242,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -5274,7 +5274,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -5306,7 +5306,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Dialogue/FirstDayIntroductionVisuals</t>
+          <t>Dialogue/CafeSceneVisuals</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -9708,7 +9708,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
     </row>
@@ -9748,7 +9748,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -9773,7 +9773,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -9803,7 +9803,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -9828,7 +9828,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -9858,7 +9858,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -9913,7 +9913,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -10063,7 +10063,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -10093,7 +10093,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -10123,7 +10123,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -10153,7 +10153,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -10178,7 +10178,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -10203,7 +10203,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -10228,7 +10228,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -10258,7 +10258,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -10283,7 +10283,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -10313,7 +10313,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -10343,7 +10343,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -10373,7 +10373,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -10403,7 +10403,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -10428,7 +10428,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -10453,7 +10453,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -10483,7 +10483,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>oct07.cafe.night</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -10513,7 +10513,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -10568,7 +10568,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -10598,7 +10598,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -10628,7 +10628,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -10653,7 +10653,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -10688,7 +10688,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -10718,7 +10718,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -10748,7 +10748,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -10778,7 +10778,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -10808,7 +10808,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -10843,7 +10843,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -10873,7 +10873,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -10903,7 +10903,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -10933,7 +10933,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -10963,7 +10963,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -10993,7 +10993,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -11053,7 +11053,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -11128,7 +11128,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -11158,7 +11158,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -11548,7 +11548,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>oct07.cafe.day</t>
+          <t>scene.cafe</t>
         </is>
       </c>
     </row>
@@ -45799,7 +45799,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>entry=Immediate;blocksSave=true;blockedBy=C-B01,C-B02,C-B05,C-G04</t>
+          <t>entry=Immediate;blocksSave=true</t>
         </is>
       </c>
     </row>
@@ -45849,7 +45849,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>entry=BeforeNight;blocksSave=true;blockedBy=C-B05,C-B06,C-G07</t>
+          <t>entry=BeforeNight;blocksSave=true</t>
         </is>
       </c>
     </row>
@@ -45899,7 +45899,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>entry=MorningBeforeMap;blocksSave=true;blockedBy=C-B03,C-B04,C-B05,B-real-completion,C-G02,C-G07</t>
+          <t>entry=MorningBeforeMap;blocksSave=true</t>
         </is>
       </c>
     </row>
@@ -45949,7 +45949,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>entry=Immediate;blocksSave=true;blockedBy=D-B03-rose-real-completion</t>
+          <t>entry=Immediate;blocksSave=true</t>
         </is>
       </c>
     </row>
@@ -46059,7 +46059,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>entry=MorningBeforeMap;blocksSave=true;blockedBy=B-B05,B-C02,B-C04,B-C07;contentBoundary=P047;previewTail=P052</t>
+          <t>entry=MorningBeforeMap;blocksSave=true;contentBoundary=P047;previewTail=P052</t>
         </is>
       </c>
     </row>
@@ -46075,7 +46075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -46308,6 +46308,54 @@
         <v>0</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>church.1009.s2</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>once</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>revolution.1013.s2</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>noon</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>once</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -46320,7 +46368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -47498,6 +47546,41 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>rose.1011.s1.complete</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>rose.1011.s1</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SET_FLAG</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>story.rose.1011.s1.completed</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Formal root completion; commit only after full presentation and reading return.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -47509,7 +47592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -48165,7 +48248,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>story.oct09.meeting.known</t>
+          <t>story.oct07.s2.completed</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -48830,7 +48913,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>story.oct09.meeting.known</t>
+          <t>story.oct07.s2.completed</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -48912,7 +48995,7 @@
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>rose.1011.s1.neutral_ready</t>
+          <t>rose.1011.s1.rose1009_ready</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -48935,7 +49018,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>story.neutral.1010.s1.completed</t>
+          <t>story.rose.1009.s1.completed</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -48947,7 +49030,7 @@
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>rose.1011.s1.rose1009_ready</t>
+          <t>rose.1011.s1.incomplete</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -48970,19 +49053,19 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>story.rose.1009.s1.completed</t>
+          <t>story.rose.1011.s1.completed</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>rose.1011.s1.incomplete</t>
+          <t>church.1009.s2.rose1009_ready</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -48992,7 +49075,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>rose.1011.s1</t>
+          <t>church.1009.s2</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -49005,12 +49088,47 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
+          <t>story.rose.1009.s1.completed</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>revolution.1014.s1.rose1011_ready</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>revolution.1014.s1</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>BOOL_EQ</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
           <t>story.rose.1011.s1.completed</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>false</t>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>

</xml_diff>